<commit_message>
feat(deploy): add local Milvus stack and register sources
</commit_message>
<xml_diff>
--- a/data/metadata/document_registry.xlsx
+++ b/data/metadata/document_registry.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="文档登记" sheetId="1" r:id="R92a224550efe4f5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="文档登记" sheetId="1" r:id="R02d9918512344798"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -50,7 +50,7 @@
     <x:numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <x:numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </x:numFmts>
-  <x:fonts count="22">
+  <x:fonts count="23">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -192,6 +192,12 @@
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
+      <x:name val="宋体"/>
+      <x:scheme val="minor"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF222222"/>
       <x:name val="宋体"/>
       <x:scheme val="minor"/>
     </x:font>
@@ -618,12 +624,16 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="3">
+  <x:cellXfs count="5">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6"/>
+    <x:xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="49">
     <x:cellStyle name="常规" xfId="0"/>
@@ -1169,6 +1179,276 @@
         <x:v>正文43条；PDF提取后仍需核对修订状态</x:v>
       </x:c>
     </x:row>
+    <x:row r="8" ht="100" customHeight="1">
+      <x:c r="A8" s="4" t="str">
+        <x:v>securities</x:v>
+      </x:c>
+      <x:c r="B8" s="4" t="str">
+        <x:v>证券公司风险控制指标管理办法</x:v>
+      </x:c>
+      <x:c r="C8" s="4" t="str">
+        <x:v>证监会令第34号（2008、2016、2020年修订）</x:v>
+      </x:c>
+      <x:c r="D8" s="4" t="str">
+        <x:v>中国证券监督管理委员会</x:v>
+      </x:c>
+      <x:c r="E8" s="4" t="str">
+        <x:v>https://www.csrc.gov.cn/csrc/c106256/c1653957/content.shtml</x:v>
+      </x:c>
+      <x:c r="F8" s="4"/>
+      <x:c r="G8" s="4" t="str">
+        <x:v>securities_证券公司风险控制指标管理办法.pdf</x:v>
+      </x:c>
+      <x:c r="H8" s="4" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="I8" s="4" t="str">
+        <x:v>effective</x:v>
+      </x:c>
+      <x:c r="J8" s="4" t="str">
+        <x:v>正文37条，14页；有文字层，未使用OCR；本批知识点33条。生效日期为原办法首次施行日；正文为2020年第三次修订合并文本，非修订决定施行日。时效按提供的官方规章版本登记；未把网页可访问当成穷尽性现行法证明。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="100" customHeight="1">
+      <x:c r="A9" s="4" t="str">
+        <x:v>securities</x:v>
+      </x:c>
+      <x:c r="B9" s="4" t="str">
+        <x:v>证券经纪业务管理办法</x:v>
+      </x:c>
+      <x:c r="C9" s="4" t="str">
+        <x:v>中国证券监督管理委员会令第204号（2023年）</x:v>
+      </x:c>
+      <x:c r="D9" s="4" t="str">
+        <x:v>中国证券监督管理委员会</x:v>
+      </x:c>
+      <x:c r="E9" s="4" t="str">
+        <x:v>https://www.csrc.gov.cn/csrc/c101953/c6987676/content.shtml</x:v>
+      </x:c>
+      <x:c r="F9" s="4"/>
+      <x:c r="G9" s="4" t="str">
+        <x:v>securities_证券经纪业务管理办法.pdf</x:v>
+      </x:c>
+      <x:c r="H9" s="4" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="I9" s="4" t="str">
+        <x:v>effective</x:v>
+      </x:c>
+      <x:c r="J9" s="4" t="str">
+        <x:v>正文53条，18页；有文字层，未使用OCR；本批知识点48条。204号令于2023年1月13日公布，2021年为审议年份。时效按提供的官方规章版本登记；未把网页可访问当成穷尽性现行法证明。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="100" customHeight="1">
+      <x:c r="A10" s="4" t="str">
+        <x:v>securities</x:v>
+      </x:c>
+      <x:c r="B10" s="4" t="str">
+        <x:v>上市公司信息披露管理办法</x:v>
+      </x:c>
+      <x:c r="C10" s="4" t="str">
+        <x:v>中国证券监督管理委员会令第226号（2025年）</x:v>
+      </x:c>
+      <x:c r="D10" s="4" t="str">
+        <x:v>中国证券监督管理委员会</x:v>
+      </x:c>
+      <x:c r="E10" s="4" t="str">
+        <x:v>https://www.csrc.gov.cn/csrc/c101953/c7547359/content.shtml</x:v>
+      </x:c>
+      <x:c r="F10" s="4"/>
+      <x:c r="G10" s="4" t="str">
+        <x:v>securities_上市公司信息披露管理办法.pdf</x:v>
+      </x:c>
+      <x:c r="H10" s="4" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="I10" s="4" t="str">
+        <x:v>effective</x:v>
+      </x:c>
+      <x:c r="J10" s="4" t="str">
+        <x:v>正文67条，21页；有文字层，未使用OCR；本批知识点62条。时效按提供的官方规章版本登记；未把网页可访问当成穷尽性现行法证明。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="100" customHeight="1">
+      <x:c r="A11" s="4" t="str">
+        <x:v>insurance</x:v>
+      </x:c>
+      <x:c r="B11" s="4" t="str">
+        <x:v>保险公司偿付能力管理规定</x:v>
+      </x:c>
+      <x:c r="C11" s="4" t="str">
+        <x:v>中国银行保险监督管理委员会令〔2021〕1号</x:v>
+      </x:c>
+      <x:c r="D11" s="4" t="str">
+        <x:v>中国银行保险监督管理委员会</x:v>
+      </x:c>
+      <x:c r="E11" s="4" t="str">
+        <x:v>https://www.nfra.gov.cn/cn/view/pages/governmentDetail.html?docId=962016&amp;itemId=861&amp;generaltype=1</x:v>
+      </x:c>
+      <x:c r="F11" s="4"/>
+      <x:c r="G11" s="4" t="str">
+        <x:v>insurance_保险公司偿付能力管理规定.pdf</x:v>
+      </x:c>
+      <x:c r="H11" s="4" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="I11" s="4" t="str">
+        <x:v>effective</x:v>
+      </x:c>
+      <x:c r="J11" s="4" t="str">
+        <x:v>正文34条，10页；有文字层，未使用OCR；本批知识点28条。时效按提供的官方规章版本登记；未把网页可访问当成穷尽性现行法证明。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="100" customHeight="1">
+      <x:c r="A12" s="4" t="str">
+        <x:v>insurance</x:v>
+      </x:c>
+      <x:c r="B12" s="4" t="str">
+        <x:v>保险资金运用管理办法</x:v>
+      </x:c>
+      <x:c r="C12" s="4" t="str">
+        <x:v>中国保险监督管理委员会令〔2018〕1号</x:v>
+      </x:c>
+      <x:c r="D12" s="4" t="str">
+        <x:v>中国保险监督管理委员会</x:v>
+      </x:c>
+      <x:c r="E12" s="4" t="str">
+        <x:v>https://www.nfra.gov.cn/cn/view/pages/rulesDetail.html?docId=1024949&amp;itemId=4214&amp;generaltype=1</x:v>
+      </x:c>
+      <x:c r="F12" s="4"/>
+      <x:c r="G12" s="4" t="str">
+        <x:v>insurance_保险资金运用管理办法.pdf</x:v>
+      </x:c>
+      <x:c r="H12" s="4" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="I12" s="4" t="str">
+        <x:v>effective</x:v>
+      </x:c>
+      <x:c r="J12" s="4" t="str">
+        <x:v>正文78条，22页；有文字层，未使用OCR；本批知识点71条。时效按提供的官方规章版本登记；未把网页可访问当成穷尽性现行法证明。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="100" customHeight="1">
+      <x:c r="A13" s="4" t="str">
+        <x:v>insurance</x:v>
+      </x:c>
+      <x:c r="B13" s="4" t="str">
+        <x:v>互联网保险业务监管办法</x:v>
+      </x:c>
+      <x:c r="C13" s="4" t="str">
+        <x:v>中国银行保险监督管理委员会令〔2020〕13号</x:v>
+      </x:c>
+      <x:c r="D13" s="4" t="str">
+        <x:v>中国银行保险监督管理委员会</x:v>
+      </x:c>
+      <x:c r="E13" s="4" t="str">
+        <x:v>https://www.nfra.gov.cn/cn/view/pages/governmentDetail.html?docId=949137&amp;itemId=861&amp;generaltype=1</x:v>
+      </x:c>
+      <x:c r="F13" s="4"/>
+      <x:c r="G13" s="4" t="str">
+        <x:v>insurance_互联网保险业务监管办法.pdf</x:v>
+      </x:c>
+      <x:c r="H13" s="4" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="I13" s="4" t="str">
+        <x:v>effective</x:v>
+      </x:c>
+      <x:c r="J13" s="4" t="str">
+        <x:v>正文83条，30页；有文字层，未使用OCR；本批知识点72条。第十四条PDF与官网字体措辞不一致，单列存疑。时效按提供的官方规章版本登记；未把网页可访问当成穷尽性现行法证明。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="100" customHeight="1">
+      <x:c r="A14" s="4" t="str">
+        <x:v>banking</x:v>
+      </x:c>
+      <x:c r="B14" s="4" t="str">
+        <x:v>商业银行金融资产风险分类办法</x:v>
+      </x:c>
+      <x:c r="C14" s="4" t="str">
+        <x:v>中国银行保险监督管理委员会、中国人民银行令〔2023〕1号</x:v>
+      </x:c>
+      <x:c r="D14" s="4" t="str">
+        <x:v>中国银行保险监督管理委员会、中国人民银行</x:v>
+      </x:c>
+      <x:c r="E14" s="4" t="str">
+        <x:v>https://www.nfra.gov.cn/cn/view/pages/governmentDetail.html?docId=1095372&amp;itemId=861&amp;generaltype=1</x:v>
+      </x:c>
+      <x:c r="F14" s="4"/>
+      <x:c r="G14" s="4" t="str">
+        <x:v>banking_商业银行金融资产风险分类办法.pdf</x:v>
+      </x:c>
+      <x:c r="H14" s="4" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="I14" s="4" t="str">
+        <x:v>effective</x:v>
+      </x:c>
+      <x:c r="J14" s="4" t="str">
+        <x:v>正文48条，16页；有文字层，未使用OCR；本批知识点43条。时效按提供的官方规章版本登记；未把网页可访问当成穷尽性现行法证明。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="100" customHeight="1">
+      <x:c r="A15" s="4" t="str">
+        <x:v>banking</x:v>
+      </x:c>
+      <x:c r="B15" s="4" t="str">
+        <x:v>商业银行大额风险暴露管理办法</x:v>
+      </x:c>
+      <x:c r="C15" s="4" t="str">
+        <x:v>中国银行保险监督管理委员会令〔2018〕1号</x:v>
+      </x:c>
+      <x:c r="D15" s="4" t="str">
+        <x:v>中国银行保险监督管理委员会</x:v>
+      </x:c>
+      <x:c r="E15" s="4" t="str">
+        <x:v>https://www.nfra.gov.cn/cn/view/pages/rulesDetail.html?docId=178636&amp;itemId=4214&amp;generaltype=1</x:v>
+      </x:c>
+      <x:c r="F15" s="4"/>
+      <x:c r="G15" s="4" t="str">
+        <x:v>banking_商业银行大额风险暴露管理办法.pdf</x:v>
+      </x:c>
+      <x:c r="H15" s="4" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="I15" s="4" t="str">
+        <x:v>effective</x:v>
+      </x:c>
+      <x:c r="J15" s="4" t="str">
+        <x:v>正文47条，23页；有文字层，未使用OCR；本批知识点37条。PDF含附件1—6，另列附件证据；附件6为历史过渡要求。时效按提供的官方规章版本登记；未把网页可访问当成穷尽性现行法证明。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="100" customHeight="1">
+      <x:c r="A16" s="4" t="str">
+        <x:v>banking</x:v>
+      </x:c>
+      <x:c r="B16" s="4" t="str">
+        <x:v>商业银行理财业务监督管理办法</x:v>
+      </x:c>
+      <x:c r="C16" s="4" t="str">
+        <x:v>中国银行保险监督管理委员会令〔2018〕6号</x:v>
+      </x:c>
+      <x:c r="D16" s="4" t="str">
+        <x:v>中国银行保险监督管理委员会</x:v>
+      </x:c>
+      <x:c r="E16" s="4" t="str">
+        <x:v>https://www.nfra.gov.cn/cn/view/pages/rulesDetail.html?docId=268592&amp;itemId=4214&amp;generaltype=1</x:v>
+      </x:c>
+      <x:c r="F16" s="4"/>
+      <x:c r="G16" s="4" t="str">
+        <x:v>banking_商业银行理财业务监督管理办法.pdf</x:v>
+      </x:c>
+      <x:c r="H16" s="4" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="I16" s="4" t="str">
+        <x:v>effective</x:v>
+      </x:c>
+      <x:c r="J16" s="4" t="str">
+        <x:v>正文81条，33页；有文字层，未使用OCR；本批知识点74条。自公布日2018-09-26施行；PDF未含第七十八条所指《商业银行理财产品销售管理要求》附件，未补写附件细节。时效按提供的官方规章版本登记；未把网页可访问当成穷尽性现行法证明。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="I2:I1000">
@@ -1176,7 +1456,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="R1b21977e537c49e7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="Rea61476b282d43e1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>